<commit_message>
added SMA 3d models, cleaned folder and added system diagram to schematic
</commit_message>
<xml_diff>
--- a/BOMs/Sample-BOM_JLCSMT.xlsx
+++ b/BOMs/Sample-BOM_JLCSMT.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="172">
   <si>
     <t xml:space="preserve">Designator</t>
   </si>
@@ -446,6 +446,15 @@
   </si>
   <si>
     <t xml:space="preserve">REF3030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIC920YC5-TR:SOT65P210X110-5N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIC920YC5-TR</t>
   </si>
   <si>
     <t xml:space="preserve">U8,U9,U10,U11</t>
@@ -563,6 +572,7 @@
       <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -576,6 +586,7 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -688,7 +699,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ559"/>
+  <dimension ref="A1:AMJ1048576"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="20" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.39"/>
@@ -1385,10 +1396,10 @@
       <c r="A62" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="0" t="s">
         <v>143</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="C62" s="5" t="s">
         <v>144</v>
       </c>
     </row>
@@ -1481,9 +1492,15 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="7"/>
-      <c r="B71" s="8"/>
-      <c r="C71" s="7"/>
+      <c r="A71" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="7"/>
@@ -3925,6 +3942,13 @@
       <c r="B559" s="8"/>
       <c r="C559" s="7"/>
     </row>
+    <row r="560" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A560" s="7"/>
+      <c r="B560" s="8"/>
+      <c r="C560" s="7"/>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>